<commit_message>
Agregar nuevos docentes: Cristian Rodriguez y Yuli Espinosa
</commit_message>
<xml_diff>
--- a/docentes.xlsx
+++ b/docentes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/556dfc19990209c2/Desktop/SAU/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniagustinianaeduco-my.sharepoint.com/personal/an_sistemasdeinformacion_uniagustiniana_edu_co/Documents/Escritorio/CREDU/CREDU/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1EB7F30E-510C-4D58-9EAB-3D9C7F468336}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="8_{1EB7F30E-510C-4D58-9EAB-3D9C7F468336}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9338560C-2FB6-42B8-A9E0-1D20F1EC1BC3}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8424" xr2:uid="{ECDFFBB1-017C-4846-ACEF-FD7E4314C05D}"/>
+    <workbookView xWindow="28680" yWindow="945" windowWidth="29040" windowHeight="15720" xr2:uid="{ECDFFBB1-017C-4846-ACEF-FD7E4314C05D}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8575" uniqueCount="4691">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8596" uniqueCount="4702">
   <si>
     <t>CEDULA</t>
   </si>
@@ -14098,6 +14098,39 @@
   </si>
   <si>
     <t>diana.rocio@uniagustiniana.edu.co</t>
+  </si>
+  <si>
+    <t>A*b79Sd*77d+b</t>
+  </si>
+  <si>
+    <t>Orrego</t>
+  </si>
+  <si>
+    <t>Lina Maria Orrego Rojas</t>
+  </si>
+  <si>
+    <t>lina.orrego@uniagustiniana.edu.co</t>
+  </si>
+  <si>
+    <t>C*l91Nc-25a/g</t>
+  </si>
+  <si>
+    <t>Cristian Fernando Rodriguez Alvarez</t>
+  </si>
+  <si>
+    <t>cristian.rodrigueza@uniagustiniana.edu.co</t>
+  </si>
+  <si>
+    <t>CO+u99Pu-80S+</t>
+  </si>
+  <si>
+    <t>Samary</t>
+  </si>
+  <si>
+    <t>Yuli Samary Espinosa Diaz</t>
+  </si>
+  <si>
+    <t>yuli.espinosa@uniagustiniana.edu.co</t>
   </si>
 </sst>
 </file>
@@ -14247,7 +14280,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -14366,12 +14399,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -14457,46 +14505,17 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="13">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -14795,13 +14814,6 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -14814,6 +14826,47 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
       </border>
     </dxf>
   </dxfs>
@@ -14830,27 +14883,27 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ADA179AA-81E9-401B-95F4-DAE7F4A65349}" name="BaseDatosSAU" displayName="BaseDatosSAU" ref="A1:I1122" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="11" tableBorderDxfId="12" totalsRowBorderDxfId="10">
-  <autoFilter ref="A1:I1122" xr:uid="{7CB83306-F00C-4F64-81D7-22D0BD0D5E6D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ADA179AA-81E9-401B-95F4-DAE7F4A65349}" name="BaseDatosSAU" displayName="BaseDatosSAU" ref="A1:I1125" totalsRowShown="0" headerRowDxfId="12" headerRowBorderDxfId="11" tableBorderDxfId="10" totalsRowBorderDxfId="9">
+  <autoFilter ref="A1:I1125" xr:uid="{7CB83306-F00C-4F64-81D7-22D0BD0D5E6D}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{F580EA34-E915-4E04-9331-399C4C23745B}" name="CEDULA" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{58A537DE-5045-4737-A35A-EC603775C7AE}" name="CONTRASEÑA" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{66BB3EF1-63E9-4F29-AE20-F163F6D7F7F5}" name="NOMBRE 1" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{9952873A-F864-435D-8033-132BA4D2256A}" name="NOMBRE 2" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{48C9D96A-00AF-4A35-89F5-5A5EC93B60A6}" name="APELLIDO 1" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{0CC4912E-1DF5-4116-A865-47E97D6681A9}" name="APELLIDO 2" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{E5F4007D-F62A-4D02-A7A6-0127E9196445}" name="NOMBRE COMPLETO" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{2963C537-F66B-414A-B73F-5DBB00D512DA}" name="LDAP" dataDxfId="2"/>
-    <tableColumn id="9" xr3:uid="{BAE592F6-37CC-410A-BE1F-FFFC321EF7A6}" name="CORREO INSTITUCIONAL" dataDxfId="1" dataCellStyle="Hipervínculo"/>
+    <tableColumn id="1" xr3:uid="{F580EA34-E915-4E04-9331-399C4C23745B}" name="CEDULA" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{58A537DE-5045-4737-A35A-EC603775C7AE}" name="CONTRASEÑA" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{66BB3EF1-63E9-4F29-AE20-F163F6D7F7F5}" name="NOMBRE 1" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{9952873A-F864-435D-8033-132BA4D2256A}" name="NOMBRE 2" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{48C9D96A-00AF-4A35-89F5-5A5EC93B60A6}" name="APELLIDO 1" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{0CC4912E-1DF5-4116-A865-47E97D6681A9}" name="APELLIDO 2" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{E5F4007D-F62A-4D02-A7A6-0127E9196445}" name="NOMBRE COMPLETO" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{2963C537-F66B-414A-B73F-5DBB00D512DA}" name="LDAP" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{BAE592F6-37CC-410A-BE1F-FFFC321EF7A6}" name="CORREO INSTITUCIONAL" dataDxfId="0" dataCellStyle="Hipervínculo"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -14888,7 +14941,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -14994,7 +15047,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -15136,7 +15189,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -15144,16 +15197,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{030B7163-AC63-43C8-87E2-58F47142DAEE}">
-  <dimension ref="A1:I1122"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <dimension ref="A1:I1125"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.109375" customWidth="1"/>
-    <col min="2" max="2" width="16.44140625" customWidth="1"/>
+    <col min="1" max="1" width="16.140625" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="6" width="12.5546875" customWidth="1"/>
-    <col min="7" max="7" width="20.5546875" customWidth="1"/>
-    <col min="9" max="9" width="39.33203125" customWidth="1"/>
+    <col min="5" max="6" width="12.5703125" customWidth="1"/>
+    <col min="7" max="7" width="20.5703125" customWidth="1"/>
+    <col min="9" max="9" width="39.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -19586,7 +19639,7 @@
         <v>844</v>
       </c>
     </row>
-    <row r="157" spans="1:9" ht="28.8">
+    <row r="157" spans="1:9">
       <c r="A157" s="23">
         <v>51987410</v>
       </c>
@@ -20991,7 +21044,7 @@
         <v>1070</v>
       </c>
     </row>
-    <row r="206" spans="1:9" ht="28.8">
+    <row r="206" spans="1:9">
       <c r="A206" s="22">
         <v>52478309</v>
       </c>
@@ -22504,7 +22557,7 @@
         <v>1310</v>
       </c>
     </row>
-    <row r="259" spans="1:9" ht="28.8">
+    <row r="259" spans="1:9">
       <c r="A259" s="22">
         <v>52918228</v>
       </c>
@@ -22674,7 +22727,7 @@
         <v>1335</v>
       </c>
     </row>
-    <row r="265" spans="1:9" ht="13.8" customHeight="1">
+    <row r="265" spans="1:9" ht="13.9" customHeight="1">
       <c r="A265" s="22">
         <v>52976134</v>
       </c>
@@ -22701,7 +22754,7 @@
         <v>1338</v>
       </c>
     </row>
-    <row r="266" spans="1:9" ht="17.399999999999999" customHeight="1">
+    <row r="266" spans="1:9" ht="17.45" customHeight="1">
       <c r="A266" s="22">
         <v>52979886</v>
       </c>
@@ -26564,7 +26617,7 @@
         <v>1919</v>
       </c>
     </row>
-    <row r="401" spans="1:9" ht="28.8">
+    <row r="401" spans="1:9">
       <c r="A401" s="22">
         <v>79611756</v>
       </c>
@@ -36148,7 +36201,7 @@
         <v>3247</v>
       </c>
     </row>
-    <row r="735" spans="1:9" ht="28.8">
+    <row r="735" spans="1:9">
       <c r="A735" s="22">
         <v>1020743419</v>
       </c>
@@ -43467,7 +43520,7 @@
         <v>4228</v>
       </c>
     </row>
-    <row r="994" spans="1:9" ht="57.6">
+    <row r="994" spans="1:9">
       <c r="A994" s="29">
         <v>1019124082</v>
       </c>
@@ -43492,7 +43545,7 @@
         <v>4232</v>
       </c>
     </row>
-    <row r="995" spans="1:9" ht="43.2">
+    <row r="995" spans="1:9">
       <c r="A995" s="29">
         <v>80793463</v>
       </c>
@@ -43735,7 +43788,7 @@
         <v>4260</v>
       </c>
     </row>
-    <row r="1004" spans="1:9" ht="43.2">
+    <row r="1004" spans="1:9">
       <c r="A1004" s="29">
         <v>73182300</v>
       </c>
@@ -43816,7 +43869,7 @@
         <v>4273</v>
       </c>
     </row>
-    <row r="1007" spans="1:9" ht="57.6">
+    <row r="1007" spans="1:9">
       <c r="A1007" s="29">
         <v>1024578317</v>
       </c>
@@ -43870,7 +43923,7 @@
         <v>4282</v>
       </c>
     </row>
-    <row r="1009" spans="1:9" ht="57.6">
+    <row r="1009" spans="1:9">
       <c r="A1009" s="29">
         <v>1032375547</v>
       </c>
@@ -43897,7 +43950,7 @@
         <v>4286</v>
       </c>
     </row>
-    <row r="1010" spans="1:9" ht="43.2">
+    <row r="1010" spans="1:9">
       <c r="A1010" s="29">
         <v>1233497048</v>
       </c>
@@ -43951,7 +44004,7 @@
         <v>4292</v>
       </c>
     </row>
-    <row r="1012" spans="1:9" ht="43.2">
+    <row r="1012" spans="1:9">
       <c r="A1012" s="29">
         <v>4431946</v>
       </c>
@@ -44057,7 +44110,7 @@
         <v>4305</v>
       </c>
     </row>
-    <row r="1016" spans="1:9" ht="43.2">
+    <row r="1016" spans="1:9">
       <c r="A1016" s="29">
         <v>80226938</v>
       </c>
@@ -44188,7 +44241,7 @@
         <v>4324</v>
       </c>
     </row>
-    <row r="1021" spans="1:9" ht="43.2">
+    <row r="1021" spans="1:9">
       <c r="A1021" s="29">
         <v>1136887283</v>
       </c>
@@ -44269,7 +44322,7 @@
         <v>4333</v>
       </c>
     </row>
-    <row r="1024" spans="1:9" ht="43.2">
+    <row r="1024" spans="1:9">
       <c r="A1024" s="29">
         <v>80831022</v>
       </c>
@@ -44350,7 +44403,7 @@
         <v>4341</v>
       </c>
     </row>
-    <row r="1027" spans="1:9" ht="57.6">
+    <row r="1027" spans="1:9">
       <c r="A1027" s="29">
         <v>1022402024</v>
       </c>
@@ -44404,7 +44457,7 @@
         <v>4348</v>
       </c>
     </row>
-    <row r="1029" spans="1:9" ht="43.2">
+    <row r="1029" spans="1:9">
       <c r="A1029" s="29">
         <v>1023916584</v>
       </c>
@@ -45535,7 +45588,7 @@
         <v>4510</v>
       </c>
     </row>
-    <row r="1072" spans="1:9" ht="55.8">
+    <row r="1072" spans="1:9">
       <c r="A1072" s="23">
         <v>1014245213</v>
       </c>
@@ -45589,7 +45642,7 @@
         <v>4519</v>
       </c>
     </row>
-    <row r="1074" spans="1:9" ht="55.8">
+    <row r="1074" spans="1:9">
       <c r="A1074" s="23">
         <v>1022431897</v>
       </c>
@@ -46888,6 +46941,87 @@
       <c r="H1122" s="41"/>
       <c r="I1122" s="42" t="s">
         <v>4690</v>
+      </c>
+    </row>
+    <row r="1123" spans="1:9">
+      <c r="A1123" s="40">
+        <v>1015412338</v>
+      </c>
+      <c r="B1123" s="43" t="s">
+        <v>4691</v>
+      </c>
+      <c r="C1123" s="43" t="s">
+        <v>588</v>
+      </c>
+      <c r="D1123" s="43" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1123" s="43" t="s">
+        <v>4692</v>
+      </c>
+      <c r="F1123" s="43" t="s">
+        <v>643</v>
+      </c>
+      <c r="G1123" s="44" t="s">
+        <v>4693</v>
+      </c>
+      <c r="H1123" s="41"/>
+      <c r="I1123" s="45" t="s">
+        <v>4694</v>
+      </c>
+    </row>
+    <row r="1124" spans="1:9">
+      <c r="A1124" s="40">
+        <v>1015433352</v>
+      </c>
+      <c r="B1124" s="43" t="s">
+        <v>4695</v>
+      </c>
+      <c r="C1124" s="43" t="s">
+        <v>2943</v>
+      </c>
+      <c r="D1124" s="43" t="s">
+        <v>261</v>
+      </c>
+      <c r="E1124" s="43" t="s">
+        <v>197</v>
+      </c>
+      <c r="F1124" s="43" t="s">
+        <v>1138</v>
+      </c>
+      <c r="G1124" s="44" t="s">
+        <v>4696</v>
+      </c>
+      <c r="H1124" s="41"/>
+      <c r="I1124" s="45" t="s">
+        <v>4697</v>
+      </c>
+    </row>
+    <row r="1125" spans="1:9">
+      <c r="A1125" s="40">
+        <v>37551633</v>
+      </c>
+      <c r="B1125" s="43" t="s">
+        <v>4698</v>
+      </c>
+      <c r="C1125" s="43" t="s">
+        <v>3032</v>
+      </c>
+      <c r="D1125" s="43" t="s">
+        <v>4699</v>
+      </c>
+      <c r="E1125" s="43" t="s">
+        <v>1895</v>
+      </c>
+      <c r="F1125" s="43" t="s">
+        <v>181</v>
+      </c>
+      <c r="G1125" s="44" t="s">
+        <v>4700</v>
+      </c>
+      <c r="H1125" s="41"/>
+      <c r="I1125" s="45" t="s">
+        <v>4701</v>
       </c>
     </row>
   </sheetData>
@@ -46951,10 +47085,13 @@
     <hyperlink ref="I1120" r:id="rId57" display="mailto:jorge.munoz@uniagustiniana.edu.co" xr:uid="{49859E95-2A87-4998-8DD6-E6FF7E3CBF45}"/>
     <hyperlink ref="I1121" r:id="rId58" display="mailto:carolina.romero@uniagustiniana.edu.co" xr:uid="{6573B2F3-ABD2-4DF1-AD8E-EAE640E9A50B}"/>
     <hyperlink ref="I1122" r:id="rId59" display="mailto:diana.rocio@uniagustiniana.edu.co" xr:uid="{B6386F8E-8059-4EB2-8406-E9D7E286B527}"/>
+    <hyperlink ref="I1123" r:id="rId60" display="mailto:lina.orrego@uniagustiniana.edu.co" xr:uid="{3148B547-02E5-4A1A-9892-06BD5753BED0}"/>
+    <hyperlink ref="I1124" r:id="rId61" display="mailto:cristian.rodrigueza@uniagustiniana.edu.co" xr:uid="{0F4F44CE-8321-41E9-80F3-B3CA7B3F54DD}"/>
+    <hyperlink ref="I1125" r:id="rId62" display="mailto:yuli.espinosa@uniagustiniana.edu.co" xr:uid="{C6727EBD-E58F-42AE-9A84-946E9D9637BC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId60"/>
+    <tablePart r:id="rId63"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualizar lista de docentes
</commit_message>
<xml_diff>
--- a/docentes.xlsx
+++ b/docentes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniagustinianaeduco-my.sharepoint.com/personal/an_sistemasdeinformacion_uniagustiniana_edu_co/Documents/Escritorio/CREDU/CREDU/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="8_{1EB7F30E-510C-4D58-9EAB-3D9C7F468336}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9338560C-2FB6-42B8-A9E0-1D20F1EC1BC3}"/>
+  <xr:revisionPtr revIDLastSave="48" documentId="8_{1EB7F30E-510C-4D58-9EAB-3D9C7F468336}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B1635C8-27B7-44A9-967D-5B56143A117C}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="945" windowWidth="29040" windowHeight="15720" xr2:uid="{ECDFFBB1-017C-4846-ACEF-FD7E4314C05D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8596" uniqueCount="4702">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8617" uniqueCount="4711">
   <si>
     <t>CEDULA</t>
   </si>
@@ -14131,6 +14131,33 @@
   </si>
   <si>
     <t>yuli.espinosa@uniagustiniana.edu.co</t>
+  </si>
+  <si>
+    <t>M*z71Be+52n+g</t>
+  </si>
+  <si>
+    <t>Adriana Carolina Perez Cortes</t>
+  </si>
+  <si>
+    <t>adriana.perez@uniagustiniana.edu.co</t>
+  </si>
+  <si>
+    <t>/27nW+j60Nx48x</t>
+  </si>
+  <si>
+    <t>Jairo Segundo Gomez Barrera</t>
+  </si>
+  <si>
+    <t>jairo.gomez@uniagustiniana.edu.co</t>
+  </si>
+  <si>
+    <t>KU/e95Uu*71K/</t>
+  </si>
+  <si>
+    <t>Francisco Javier Rodriguez Quiroga</t>
+  </si>
+  <si>
+    <t>francisco.rodriguez@uniagustiniana.edu.co</t>
   </si>
 </sst>
 </file>
@@ -14419,7 +14446,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -14510,6 +14537,10 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -14882,9 +14913,13 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ADA179AA-81E9-401B-95F4-DAE7F4A65349}" name="BaseDatosSAU" displayName="BaseDatosSAU" ref="A1:I1125" totalsRowShown="0" headerRowDxfId="12" headerRowBorderDxfId="11" tableBorderDxfId="10" totalsRowBorderDxfId="9">
-  <autoFilter ref="A1:I1125" xr:uid="{7CB83306-F00C-4F64-81D7-22D0BD0D5E6D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ADA179AA-81E9-401B-95F4-DAE7F4A65349}" name="BaseDatosSAU" displayName="BaseDatosSAU" ref="A1:I1128" totalsRowShown="0" headerRowDxfId="12" headerRowBorderDxfId="11" tableBorderDxfId="10" totalsRowBorderDxfId="9">
+  <autoFilter ref="A1:I1128" xr:uid="{7CB83306-F00C-4F64-81D7-22D0BD0D5E6D}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{F580EA34-E915-4E04-9331-399C4C23745B}" name="CEDULA" dataDxfId="8"/>
     <tableColumn id="2" xr3:uid="{58A537DE-5045-4737-A35A-EC603775C7AE}" name="CONTRASEÑA" dataDxfId="7"/>
@@ -15197,7 +15232,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{030B7163-AC63-43C8-87E2-58F47142DAEE}">
-  <dimension ref="A1:I1125"/>
+  <dimension ref="A1:I1128"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16.140625" customWidth="1"/>
@@ -47022,6 +47057,87 @@
       <c r="H1125" s="41"/>
       <c r="I1125" s="45" t="s">
         <v>4701</v>
+      </c>
+    </row>
+    <row r="1126" spans="1:9">
+      <c r="A1126" s="40">
+        <v>1018424897</v>
+      </c>
+      <c r="B1126" s="43" t="s">
+        <v>4702</v>
+      </c>
+      <c r="C1126" s="43" t="s">
+        <v>841</v>
+      </c>
+      <c r="D1126" s="43" t="s">
+        <v>601</v>
+      </c>
+      <c r="E1126" s="43" t="s">
+        <v>58</v>
+      </c>
+      <c r="F1126" s="43" t="s">
+        <v>512</v>
+      </c>
+      <c r="G1126" s="44" t="s">
+        <v>4703</v>
+      </c>
+      <c r="H1126" s="41"/>
+      <c r="I1126" s="46" t="s">
+        <v>4704</v>
+      </c>
+    </row>
+    <row r="1127" spans="1:9">
+      <c r="A1127" s="40">
+        <v>79975194</v>
+      </c>
+      <c r="B1127" s="43" t="s">
+        <v>4705</v>
+      </c>
+      <c r="C1127" s="43" t="s">
+        <v>139</v>
+      </c>
+      <c r="D1127" s="43" t="s">
+        <v>206</v>
+      </c>
+      <c r="E1127" s="43" t="s">
+        <v>314</v>
+      </c>
+      <c r="F1127" s="47" t="s">
+        <v>2134</v>
+      </c>
+      <c r="G1127" s="44" t="s">
+        <v>4706</v>
+      </c>
+      <c r="H1127" s="41"/>
+      <c r="I1127" s="45" t="s">
+        <v>4707</v>
+      </c>
+    </row>
+    <row r="1128" spans="1:9">
+      <c r="A1128" s="40">
+        <v>80065613</v>
+      </c>
+      <c r="B1128" s="43" t="s">
+        <v>4708</v>
+      </c>
+      <c r="C1128" s="43" t="s">
+        <v>178</v>
+      </c>
+      <c r="D1128" s="43" t="s">
+        <v>487</v>
+      </c>
+      <c r="E1128" s="43" t="s">
+        <v>197</v>
+      </c>
+      <c r="F1128" s="43" t="s">
+        <v>3732</v>
+      </c>
+      <c r="G1128" s="44" t="s">
+        <v>4709</v>
+      </c>
+      <c r="H1128" s="41"/>
+      <c r="I1128" s="45" t="s">
+        <v>4710</v>
       </c>
     </row>
   </sheetData>
@@ -47088,10 +47204,13 @@
     <hyperlink ref="I1123" r:id="rId60" display="mailto:lina.orrego@uniagustiniana.edu.co" xr:uid="{3148B547-02E5-4A1A-9892-06BD5753BED0}"/>
     <hyperlink ref="I1124" r:id="rId61" display="mailto:cristian.rodrigueza@uniagustiniana.edu.co" xr:uid="{0F4F44CE-8321-41E9-80F3-B3CA7B3F54DD}"/>
     <hyperlink ref="I1125" r:id="rId62" display="mailto:yuli.espinosa@uniagustiniana.edu.co" xr:uid="{C6727EBD-E58F-42AE-9A84-946E9D9637BC}"/>
+    <hyperlink ref="I1127" r:id="rId63" display="mailto:jairo.gomez@uniagustiniana.edu.co" xr:uid="{FA3F1D34-0B35-45CC-8A5E-572A173BAFB1}"/>
+    <hyperlink ref="I1128" r:id="rId64" display="mailto:francisco.rodriguez@uniagustiniana.edu.co" xr:uid="{206FBFDE-C724-4FAC-A7B2-92C69C9650F0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId65"/>
   <tableParts count="1">
-    <tablePart r:id="rId63"/>
+    <tablePart r:id="rId66"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>